<commit_message>
Finalize Lumbee/RIVR Tech IRU package: model, README, QA, sources
- 30-year financial model (19 worksheets, formula-driven, 3 switches, 12 checks)
- README.md project index (deliverables, review order, open decisions,
  placeholder + model instructions)
- Consistency checks pass 12/0/0; injected parties line into all workbooks
- PDF conversion documented (LibreOffice non-functional in build sandbox)
- 34 deliverables across 9 subfolders

DRAFT FOR DISCUSSION – SUBJECT TO LEGAL, GRANT AND FINANCIAL REVIEW.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhaKeVxjNyTBn6poC6zJrZ
</commit_message>
<xml_diff>
--- a/Lumbee_RIVR_Tech_IRU_Package/03_Operational_Schedules/Exhibit_B_Asset_Ownership_and_Demarcation_Matrix.xlsx
+++ b/Lumbee_RIVR_Tech_IRU_Package/03_Operational_Schedules/Exhibit_B_Asset_Ownership_and_Demarcation_Matrix.xlsx
@@ -600,6 +600,14 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Parties: Lumbee Tribe of North Carolina (the “Tribe”) and LREMC Technologies, LLC d/b/a RIVR Tech (“RIVR Tech”)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -707,6 +715,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rename defined party term 'Tribe' to 'Lumbee Tribe' across package
- common.py: TRIBE_SHORT now 'Lumbee Tribe'
- Guarded rename in all generators (preserves 'Tribal' adjective, full name,
  and TRIBE_* constants); regenerated all 34 documents
- README + Sources updated; consistency check 12 PASS / 0 WARN / 0 FAIL
- Added finish_workbooks.py (parties-line injection finisher)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhaKeVxjNyTBn6poC6zJrZ
</commit_message>
<xml_diff>
--- a/Lumbee_RIVR_Tech_IRU_Package/03_Operational_Schedules/Exhibit_B_Asset_Ownership_and_Demarcation_Matrix.xlsx
+++ b/Lumbee_RIVR_Tech_IRU_Package/03_Operational_Schedules/Exhibit_B_Asset_Ownership_and_Demarcation_Matrix.xlsx
@@ -603,7 +603,7 @@
     <row r="3">
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Parties: Lumbee Tribe of North Carolina (the “Tribe”) and LREMC Technologies, LLC d/b/a RIVR Tech (“RIVR Tech”)</t>
+          <t>Parties: Lumbee Tribe of North Carolina (the “Lumbee Tribe”) and LREMC Technologies, LLC d/b/a RIVR Tech (“RIVR Tech”)</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>• Grant-funded Tribal Assets are owned by the Tribe and carry a Federal Interest (YES) under 2 CFR 200.313 and the property-trust relationship of 2 CFR 200.316.</t>
+          <t>• Grant-funded Tribal Assets are owned by the Lumbee Tribe and carry a Federal Interest (YES) under 2 CFR 200.313 and the property-trust relationship of 2 CFR 200.316.</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Owner (Tribe/RIVR Tech/Joint)</t>
+          <t>Owner (Lumbee Tribe/RIVR Tech/Joint)</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Tribe</t>
+          <t>Lumbee Tribe</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>[■ Tribe / RIVR Tech / Joint]</t>
+          <t>[■ Lumbee Tribe / RIVR Tech / Joint]</t>
         </is>
       </c>
       <c r="E19" s="16" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>[■ Tribe / RIVR Tech / pole owner]</t>
+          <t>[■ Lumbee Tribe / RIVR Tech / pole owner]</t>
         </is>
       </c>
       <c r="E20" s="16" t="inlineStr">
@@ -1498,7 +1498,7 @@
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>• The Demarcation Point is the physical (or logical) boundary at which ownership, operational control, maintenance responsibility, and risk of loss pass between the Tribe (Tribal Assets) and RIVR Tech (RIVR Tech Existing Network / core).</t>
+          <t>• The Demarcation Point is the physical (or logical) boundary at which ownership, operational control, maintenance responsibility, and risk of loss pass between the Lumbee Tribe (Tribal Assets) and RIVR Tech (RIVR Tech Existing Network / core).</t>
         </is>
       </c>
       <c r="B25" s="18" t="n"/>
@@ -1512,7 +1512,7 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>• On the Tribe's side of each Demarcation Point the plant is a grant-funded Tribal Asset subject to the Federal Interest and the property-trust relationship (2 CFR 200.316) until disposition per 2 CFR 200.313.</t>
+          <t>• On the Lumbee Tribe's side of each Demarcation Point the plant is a grant-funded Tribal Asset subject to the Federal Interest and the property-trust relationship (2 CFR 200.316) until disposition per 2 CFR 200.313.</t>
         </is>
       </c>
       <c r="B26" s="18" t="n"/>

</xml_diff>